<commit_message>
fix: şık metinlerinden PDF açıklamalarını temizle (131 düzeltme)
21-22 Final/Bütünleme ve 22-23 Yaz Okulu sınavlarının PDF'lerinde
her sorudan sonra gelen 'Cevap Açıklama:' metinleri extraction
sırasında son şıklara karışmıştı. 6 ders × tüm sınavlar yeniden
extract edilip 131 şık düzeltildi, HTML sayfaları güncellendi.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/1_sinif/bahar/Dosyalama_ve_Arsivleme_Soru_Bankasi.xlsx
+++ b/1_sinif/bahar/Dosyalama_ve_Arsivleme_Soru_Bankasi.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,56 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001B5E3A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001E3A8A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00065F46"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="007A5800"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="009A3412"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00444444"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -82,48 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -580,7 +504,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Şehir arşivi tarandan kullanılan arşivleme sisteminde, birbirlerinden bağımsız olarak faaliyet gösteren arşivler dağınık arşivlerdir.</t>
+          <t>Şehir arşivi</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -625,7 +549,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>%60-70 alanlarda higrometre bulundurmak sureyle, rutuben %50-60 arasında tutulmasının sağlanması gerekmektedir.</t>
+          <t>%60-70</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -670,7 +594,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Belge numarası verme gerçekleşrilen bir faaliyet değildir.</t>
+          <t>Belge numarası verme</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -700,7 +624,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Yapğı hizmetlerde ve yerine gerdiği görevlerde özveri ile çalışarak yüksek performans gösterir.</t>
+          <t>Yapğı hizmetlerde ve yerine gerdiği görevlerde özveri ile</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -715,7 +639,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Dosyalama ve arşivleme bölümüne ait çalışma ortamının düzenli ve temiz tutulması işine karışmaz. CEVAP AN</t>
+          <t>Dosyalama ve arşivleme bölümüne ait çalışma ortamının</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1345,7 +1269,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Formun kayıt edilmesi ve gerekli bilgilerin yazılabilmesi için boş alanlar içermelidir. kısa olmalıdır. CEVAP AN</t>
+          <t>Formun kayıt edilmesi ve gerekli bilgilerin yazılabilmesi için</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1435,7 +1359,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>İşletmenin kaynaklarını en etkili biçimde kullanabilmek için değişen durumlara ilişkin kısa dönemli alınan kararlardır.</t>
+          <t>İşletmenin kaynaklarını en etkili biçimde kullanabilmek için</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1615,7 +1539,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Genel arşiv kuruluşlarındaki arşivleri birim arşivi sayılır. Mükellef arşivi ve genel arşiv bulunmamaktadır.</t>
+          <t>Genel arşiv</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2020,7 +1944,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Formların çizilmesinde estek ve form tekniklerine eşit oranda önem verilmelidir. CEVAP AN</t>
+          <t>Formların çizilmesinde estek ve form tekniklerine eşit oranda</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2110,7 +2034,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Formun üst kısmında, form isim ve numarası ile formu hazırlayan kuruluşun unvanı, alt kısmında ise kullanıma başladığı tarih, stok numarası ve basım adedi yer almalıdır.</t>
+          <t>Formun üst kısmında, form isim ve numarası ile formu</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2380,7 +2304,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Arşiv malzemelerinin en üst amirin onayına sunulması fonksiyonları aşağıdaki gibi sıralanabilir. •İlgili arşiv malzemelerinin tespit edilmesi, •Arşive kaldırılan malzemelerin sınıflandırılması, •Arşiv malzemelerinin ayırılması, •Arşiv malzemelerinin kayba uğramalarının önüne geçilmesi</t>
+          <t>Arşiv malzemelerinin en üst amirin onayına sunulması</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2605,7 +2529,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Nokta yöntemi alınışında köşesine bir nokta koymayı içerir. Böylece bir evrakın gereksiz yere kaç defa ele aldığı kolaylıkla görülebilir. CEVAP AN</t>
+          <t>Nokta yöntemi</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2650,7 +2574,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Dosyanın ödünç verilmesi ve takibi yeni evrak oluşturulmaz. Oluşturulmuş evrakların dosyalama işlemlerine ve oluşturulmuş dosyalara ait süreci kapsamaktadır.</t>
+          <t>Dosyanın ödünç verilmesi ve takibi</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2740,7 +2664,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Evrak postalama ve gönderme işlerini düzenli bir şekilde yürütmeleri personeli işletme içerisinde aşağıdaki işlemleri gerçekleşrir: Evraklardaki postalama ve gönderme işlerini düzenli bir şekilde yürütmek,</t>
+          <t>Evrak postalama ve gönderme işlerini düzenli bir şekilde</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2785,7 +2709,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Düşük maliyete sahip olmalı aşamasında maliyet ana kriterler arasında yer almaz.</t>
+          <t>Düşük maliyete sahip olmalı</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2875,7 +2799,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Kutu klasör materyaldir. Bu nedenle dosyalamada kullanılan bir araç değildir.</t>
+          <t>Kutu klasör</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2965,7 +2889,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Sistemlerde uyumluluk problemlerinin ortaya çıkması birisi, Sistemlerde uyumluluk problemleri ortaya çıkmaktadır.</t>
+          <t>Sistemlerde uyumluluk problemlerinin ortaya çıkması</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3145,7 +3069,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Arşiv indekslerinin saklama ve bulma işlemlerini kolaylaşracak şekilde hazırlanması</t>
+          <t>Arşiv indekslerinin saklama ve bulma işlemlerini kolaylaşracak</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3190,7 +3114,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>İşlerin daha yüksek bir maliyetle yapılması daha az maliyetle, daha kısa sürede ve daha kolay bir şekilde yapılmasını sağlamak amacıyla tüm faaliyetlerin sistemak bir şekilde incelenmesi ve gelişrilmesidir.</t>
+          <t>İşlerin daha yüksek bir maliyetle yapılması</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3640,7 +3564,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Personelin monotonluğa sevk etmesi ücret ve unvan, daha fazla presj ve sorumluluk gerirken aşağıdaki amaçlara hizmet etmektedir:</t>
+          <t>Personelin monotonluğa sevk etmesi</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3730,7 +3654,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Dosya gömleği konulduğu ve bu dosyaları koruma, istenildiğinde erişimi kolaylaşrma amacıyla tasarlanmış dolaplara dosya dolabı denilmektedir.</t>
+          <t>Dosya gömleği</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3955,7 +3879,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Bürolar, özel sektör veya kamuda işlerin büyük bir kısmının yürütüldüğü yerlerdir.</t>
+          <t>Bürolar, özel sektör veya kamuda işlerin büyük bir kısmının</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -4000,7 +3924,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Kolluk görevlileri kullanılmasına ve muhafazasına lüzum görülmeyen her türlü malzemenin ayıklama ve imhası, kurum arşivlerinde kendilerince yapılır</t>
+          <t>Kolluk görevlileri</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -4090,7 +4014,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Dosyalama sistemlerinin hiç bir türü her duruma uygun olmadığından hangisinin daha iyi olduğunu belirlemek zordur.</t>
+          <t>Dosyalama sistemlerinin hiç bir türü her duruma uygun</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -4180,7 +4104,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Örgütleme örgütlerde dosyalama yöneminde karışıklıkların ortadan kaldırılması amaçlanmaktadır.</t>
+          <t>Örgütleme</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4315,7 +4239,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Örgütün günlük faaliyetlerinin etkin bir şekilde sürdürülmesini sağlaması ve daha detaylıdır. EBYS’ler, TSE TS 13298 ulusal standardına uygun şekilde hazırlanır. EBYS’ler gelişmiş fonksiyonlar içeren sistemlerdir</t>
+          <t>Örgütün günlük faaliyetlerinin etkin bir şekilde</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4585,7 +4509,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>I, II, III ve IV işlev ve fonksiyonları arasında yer almaktadır.</t>
+          <t>I, II, III ve IV</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4810,7 +4734,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>I, II, III ve IV dosya planının kuruma sağladığı faydalardandır.</t>
+          <t>I, II, III ve IV</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -5035,7 +4959,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Eski harfli belgelerdeki Hicri ve Rumi tarihler, Miladi tarihe çevrilerek alınır.</t>
+          <t>Eski harfli belgelerdeki Hicri ve Rumi tarihler, Miladi tarihe</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5170,7 +5094,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>5-10 yıl - 20-30 yıl malzeme, birim arşivlerinde 1-5 süre ile arşiv malzemesi ise kurum arşivlerinde10-14 yıl saklanır.</t>
+          <t>5-10 yıl - 20-30 yıl</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">

</xml_diff>

<commit_message>
fix: manuel düzeltmeler sonrası HTML'ler yeniden üretildi
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/1_sinif/bahar/Dosyalama_ve_Arsivleme_Soru_Bankasi.xlsx
+++ b/1_sinif/bahar/Dosyalama_ve_Arsivleme_Soru_Bankasi.xlsx
@@ -512,6 +512,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -557,6 +558,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -602,6 +604,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -647,6 +650,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -692,6 +696,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -737,6 +742,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -782,6 +788,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -827,6 +834,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -872,6 +880,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -917,6 +926,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -962,6 +972,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1007,6 +1018,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1052,6 +1064,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1097,6 +1110,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1142,6 +1156,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1187,6 +1202,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1232,6 +1248,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1277,6 +1294,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1322,6 +1340,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1367,6 +1386,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1412,6 +1432,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1457,6 +1478,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1502,6 +1524,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1547,6 +1570,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1592,6 +1616,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1637,6 +1662,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1682,6 +1708,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1727,6 +1754,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1772,6 +1800,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1817,6 +1846,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1862,6 +1892,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1907,6 +1938,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1952,6 +1984,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1997,6 +2030,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2042,6 +2076,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2087,6 +2122,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2132,6 +2168,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2177,6 +2214,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2222,6 +2260,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2267,6 +2306,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2312,6 +2352,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2357,6 +2398,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2402,6 +2444,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2447,6 +2490,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2492,6 +2536,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2537,6 +2582,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2582,6 +2628,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2619,7 +2666,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Kronolojik Dosyalama Sistemi CEVAP AN</t>
+          <t>Kronolojik Dosyalama Sistemi</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2627,6 +2674,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2672,6 +2720,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2717,6 +2766,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2762,6 +2812,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2807,6 +2858,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2852,6 +2904,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2897,6 +2950,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2942,6 +2996,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2987,6 +3042,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3024,7 +3080,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Yazının çoğallma sayısı CEVAP AN</t>
+          <t>Yazının çoğallma sayısı</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3032,6 +3088,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3077,6 +3134,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3122,6 +3180,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3167,6 +3226,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3212,6 +3272,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3257,6 +3318,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3302,6 +3364,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3347,6 +3410,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3392,6 +3456,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3437,6 +3502,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3482,6 +3548,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3519,7 +3586,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Emek piyasası CEVAP AN</t>
+          <t>Emek piyasası</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3527,6 +3594,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3572,6 +3640,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3617,6 +3686,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3662,6 +3732,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3707,6 +3778,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3752,6 +3824,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3797,6 +3870,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3834,7 +3908,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Rütbe indirimi CEVAP AN</t>
+          <t>Rütbe indirimi</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -3842,6 +3916,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3887,6 +3962,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3932,6 +4008,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3977,6 +4054,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -4022,6 +4100,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -4067,6 +4146,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -4112,6 +4192,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -4157,6 +4238,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -4202,6 +4284,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -4247,6 +4330,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -4292,6 +4376,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -4337,6 +4422,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -4382,6 +4468,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -4427,6 +4514,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -4472,6 +4560,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4517,6 +4606,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4562,6 +4652,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -4607,6 +4698,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -4652,6 +4744,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -4697,6 +4790,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -4742,6 +4836,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -4787,6 +4882,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -4832,6 +4928,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -4877,6 +4974,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -4922,6 +5020,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -4967,6 +5066,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -5012,6 +5112,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -5057,6 +5158,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -5102,6 +5204,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -5147,6 +5250,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -5192,6 +5296,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -5237,6 +5342,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -5282,6 +5388,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -5327,6 +5434,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -5372,6 +5480,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -5417,6 +5526,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -5462,6 +5572,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -5507,6 +5618,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -5552,6 +5664,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -5597,6 +5710,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -5642,6 +5756,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -5687,6 +5802,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -5732,6 +5848,7 @@
           <t>D</t>
         </is>
       </c>
+      <c r="J118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -5777,6 +5894,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -5822,6 +5940,7 @@
           <t>E</t>
         </is>
       </c>
+      <c r="J120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -5867,6 +5986,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -5912,6 +6032,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -5957,6 +6078,7 @@
           <t>C</t>
         </is>
       </c>
+      <c r="J123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -6002,6 +6124,7 @@
           <t>B</t>
         </is>
       </c>
+      <c r="J124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -6047,6 +6170,7 @@
           <t>A</t>
         </is>
       </c>
+      <c r="J125" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>